<commit_message>
Some minor changes included
</commit_message>
<xml_diff>
--- a/12625822.xlsx
+++ b/12625822.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LPU\sem 1\Python\CAP776\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LPU\sem 1\Python\MInor Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC9945AE-4345-49A4-AFE3-FFC936C016D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9558770-D0F8-49C3-945D-B8ABC7A2F329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="83">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -281,6 +281,9 @@
   </si>
   <si>
     <t>Played football after a long time.</t>
+  </si>
+  <si>
+    <t>Started my daily recording.</t>
   </si>
 </sst>
 </file>
@@ -1087,7 +1090,9 @@
       <c r="M6" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="N6" s="12"/>
+      <c r="N6" s="12" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
@@ -1833,7 +1838,7 @@
         <v>800</v>
       </c>
       <c r="J23" s="10">
-        <f t="shared" si="7"/>
+        <f>IF(I23="","",1440-I23)</f>
         <v>640</v>
       </c>
       <c r="K23" s="11" t="s">
@@ -1903,7 +1908,7 @@
         <v>420</v>
       </c>
       <c r="C25" s="9">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D25" s="9">
         <v>60</v>
@@ -1917,62 +1922,114 @@
       <c r="G25" s="9">
         <v>5</v>
       </c>
-      <c r="H25" s="9"/>
+      <c r="H25" s="9">
+        <v>0</v>
+      </c>
       <c r="I25" s="10">
         <f t="shared" si="6"/>
-        <v>800</v>
+        <v>810</v>
       </c>
       <c r="J25" s="10">
         <f t="shared" si="7"/>
-        <v>640</v>
-      </c>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
+        <v>630</v>
+      </c>
+      <c r="K25" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L25" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M25" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="N25" s="12"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="8">
         <v>46267</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
+      <c r="B26" s="9">
+        <v>360</v>
+      </c>
+      <c r="C26" s="9">
+        <v>80</v>
+      </c>
+      <c r="D26" s="9">
+        <v>0</v>
+      </c>
+      <c r="E26" s="9">
+        <v>0</v>
+      </c>
       <c r="F26" s="9">
         <v>200</v>
       </c>
       <c r="G26" s="9">
         <v>4</v>
       </c>
-      <c r="H26" s="9"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
+      <c r="H26" s="9">
+        <v>0</v>
+      </c>
+      <c r="I26" s="10">
+        <f t="shared" si="6"/>
+        <v>640</v>
+      </c>
+      <c r="J26" s="10">
+        <f t="shared" si="7"/>
+        <v>800</v>
+      </c>
+      <c r="K26" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L26" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M26" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N26" s="12"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="8">
         <v>46268</v>
       </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
+      <c r="B27" s="9">
+        <v>360</v>
+      </c>
+      <c r="C27" s="9">
+        <v>80</v>
+      </c>
+      <c r="D27" s="9">
+        <v>0</v>
+      </c>
+      <c r="E27" s="9">
+        <v>0</v>
+      </c>
       <c r="F27" s="9">
         <v>250</v>
       </c>
       <c r="G27" s="9">
         <v>5</v>
       </c>
-      <c r="H27" s="9"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
+      <c r="H27" s="9">
+        <v>0</v>
+      </c>
+      <c r="I27" s="10">
+        <f t="shared" si="6"/>
+        <v>690</v>
+      </c>
+      <c r="J27" s="10">
+        <f t="shared" si="7"/>
+        <v>750</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L27" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M27" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N27" s="12"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -1985,15 +2042,21 @@
       <c r="C28" s="9">
         <v>80</v>
       </c>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
+      <c r="D28" s="9">
+        <v>0</v>
+      </c>
+      <c r="E28" s="9">
+        <v>0</v>
+      </c>
       <c r="F28" s="9">
         <v>300</v>
       </c>
       <c r="G28" s="9">
         <v>6</v>
       </c>
-      <c r="H28" s="9"/>
+      <c r="H28" s="9">
+        <v>0</v>
+      </c>
       <c r="I28" s="10">
         <f t="shared" si="6"/>
         <v>720</v>
@@ -2002,9 +2065,15 @@
         <f t="shared" si="7"/>
         <v>720</v>
       </c>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
+      <c r="K28" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L28" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M28" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N28" s="12"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
@@ -2015,28 +2084,40 @@
         <v>420</v>
       </c>
       <c r="C29" s="9">
-        <v>80</v>
-      </c>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
+        <v>120</v>
+      </c>
+      <c r="D29" s="9">
+        <v>0</v>
+      </c>
+      <c r="E29" s="9">
+        <v>0</v>
+      </c>
       <c r="F29" s="9">
         <v>0</v>
       </c>
       <c r="G29" s="9">
         <v>0</v>
       </c>
-      <c r="H29" s="9"/>
+      <c r="H29" s="9">
+        <v>0</v>
+      </c>
       <c r="I29" s="10">
         <f t="shared" si="6"/>
-        <v>500</v>
+        <v>540</v>
       </c>
       <c r="J29" s="10">
         <f t="shared" si="7"/>
-        <v>940</v>
-      </c>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
+        <v>900</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L29" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M29" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="N29" s="12"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
@@ -2047,28 +2128,40 @@
         <v>440</v>
       </c>
       <c r="C30" s="9">
-        <v>80</v>
-      </c>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
+        <v>10</v>
+      </c>
+      <c r="D30" s="9">
+        <v>0</v>
+      </c>
+      <c r="E30" s="9">
+        <v>0</v>
+      </c>
       <c r="F30" s="9">
         <v>0</v>
       </c>
       <c r="G30" s="9">
         <v>0</v>
       </c>
-      <c r="H30" s="9"/>
+      <c r="H30" s="9">
+        <v>0</v>
+      </c>
       <c r="I30" s="10">
         <f t="shared" si="6"/>
-        <v>520</v>
+        <v>450</v>
       </c>
       <c r="J30" s="10">
         <f t="shared" si="7"/>
-        <v>920</v>
-      </c>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
+        <v>990</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L30" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M30" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N30" s="12"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
@@ -2081,15 +2174,21 @@
       <c r="C31" s="9">
         <v>80</v>
       </c>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
+      <c r="D31" s="9">
+        <v>0</v>
+      </c>
+      <c r="E31" s="9">
+        <v>0</v>
+      </c>
       <c r="F31" s="9">
         <v>350</v>
       </c>
       <c r="G31" s="9">
         <v>7</v>
       </c>
-      <c r="H31" s="9"/>
+      <c r="H31" s="9">
+        <v>0</v>
+      </c>
       <c r="I31" s="10">
         <f t="shared" si="6"/>
         <v>840</v>
@@ -2098,9 +2197,15 @@
         <f t="shared" si="7"/>
         <v>600</v>
       </c>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
+      <c r="K31" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L31" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M31" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N31" s="12"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
@@ -2113,15 +2218,21 @@
       <c r="C32" s="9">
         <v>80</v>
       </c>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
+      <c r="D32" s="9">
+        <v>0</v>
+      </c>
+      <c r="E32" s="9">
+        <v>0</v>
+      </c>
       <c r="F32" s="9">
         <v>250</v>
       </c>
       <c r="G32" s="9">
         <v>5</v>
       </c>
-      <c r="H32" s="9"/>
+      <c r="H32" s="9">
+        <v>0</v>
+      </c>
       <c r="I32" s="10">
         <f t="shared" si="6"/>
         <v>670</v>
@@ -2130,31 +2241,59 @@
         <f t="shared" si="7"/>
         <v>770</v>
       </c>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
+      <c r="K32" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L32" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M32" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N32" s="12"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
         <v>46274</v>
       </c>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
+      <c r="B33" s="9">
+        <v>420</v>
+      </c>
+      <c r="C33" s="9">
+        <v>80</v>
+      </c>
+      <c r="D33" s="9">
+        <v>0</v>
+      </c>
+      <c r="E33" s="9">
+        <v>0</v>
+      </c>
       <c r="F33" s="9">
         <v>200</v>
       </c>
       <c r="G33" s="9">
         <v>4</v>
       </c>
-      <c r="H33" s="9"/>
-      <c r="I33" s="10"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
+      <c r="H33" s="9">
+        <v>0</v>
+      </c>
+      <c r="I33" s="10">
+        <f t="shared" si="6"/>
+        <v>700</v>
+      </c>
+      <c r="J33" s="10">
+        <f t="shared" si="7"/>
+        <v>740</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L33" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="N33" s="12"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
@@ -2529,22 +2668,44 @@
       <c r="A42" s="8">
         <v>46283</v>
       </c>
-      <c r="B42" s="9"/>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9"/>
+      <c r="B42" s="9">
+        <v>420</v>
+      </c>
+      <c r="C42" s="9">
+        <v>80</v>
+      </c>
+      <c r="D42" s="9">
+        <v>170</v>
+      </c>
+      <c r="E42" s="9">
+        <v>50</v>
+      </c>
       <c r="F42" s="9">
         <v>300</v>
       </c>
       <c r="G42" s="9">
         <v>6</v>
       </c>
-      <c r="H42" s="9"/>
-      <c r="I42" s="10"/>
-      <c r="J42" s="10"/>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
+      <c r="H42" s="9">
+        <v>30</v>
+      </c>
+      <c r="I42" s="10">
+        <f t="shared" si="6"/>
+        <v>1050</v>
+      </c>
+      <c r="J42" s="10">
+        <f t="shared" si="7"/>
+        <v>390</v>
+      </c>
+      <c r="K42" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="L42" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="M42" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="N42" s="12"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>